<commit_message>
Complete Festify progress tracker items
</commit_message>
<xml_diff>
--- a/Software_Development_Progress_Tracker_Festify.xlsx
+++ b/Software_Development_Progress_Tracker_Festify.xlsx
@@ -149,7 +149,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
@@ -395,14 +395,14 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Belum ada proses verifikasi email setelah registrasi.</t>
+          <t>Verifikasi email aktif melalui MustVerifyEmail, route verifikasi, notice, dan kirim ulang link.</t>
         </is>
       </c>
       <c r="E9" s="6">
         <v>2</v>
       </c>
       <c r="F9" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(F9/E9,0)</f>
@@ -414,7 +414,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>MustVerifyEmail, mailable, dan route verifikasi belum diaktifkan.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -434,14 +434,14 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Belum ada fitur reset password via email.</t>
+          <t>Reset password user aktif memakai password_reset_tokens dan notifikasi reset bawaan Laravel.</t>
         </is>
       </c>
       <c r="E10" s="6">
         <v>1</v>
       </c>
       <c r="F10" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="7">
         <f>IFERROR(F10/E10,0)</f>
@@ -453,7 +453,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Route, controller, dan notifikasi reset password belum dibuat.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -746,14 +746,14 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>User memilih zona dan jumlah tiket; stok konser dan zona dikurangi dalam transaksi DB.</t>
+          <t>User memilih zona dan jumlah tiket; stok konser dan zona dikurangi dalam DB transaction dengan lockForUpdate.</t>
         </is>
       </c>
       <c r="E18" s="6">
         <v>5</v>
       </c>
       <c r="F18" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G18" s="7">
         <f>IFERROR(F18/E18,0)</f>
@@ -765,7 +765,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Belum memakai lockForUpdate sehingga masih ada risiko race condition saat traffic tinggi.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1292,14 +1292,14 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Belum ada fitur unduh laporan.</t>
+          <t>Admin dapat mengunduh laporan riwayat scan dalam format CSV.</t>
         </is>
       </c>
       <c r="E32" s="6">
         <v>1</v>
       </c>
       <c r="F32" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="7">
         <f>IFERROR(F32/E32,0)</f>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Belum ada endpoint export dan library seperti Laravel Excel/DomPDF.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1331,14 +1331,14 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Dashboard menampilkan jumlah e-ticket ditukar dan gelang aktif.</t>
+          <t>Dashboard menampilkan jumlah e-ticket ditukar, gelang aktif, dan 8 riwayat scan terakhir.</t>
         </is>
       </c>
       <c r="E33" s="6">
         <v>3</v>
       </c>
       <c r="F33" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33" s="7">
         <f>IFERROR(F33/E33,0)</f>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Belum menampilkan riwayat scan terakhir langsung di dashboard.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1409,14 +1409,14 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Dashboard menampilkan jumlah gelang sudah masuk dan gelang aktif.</t>
+          <t>Dashboard menampilkan jumlah gelang masuk, gelang aktif, dan 8 riwayat scan terakhir.</t>
         </is>
       </c>
       <c r="E35" s="6">
         <v>3</v>
       </c>
       <c r="F35" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" s="7">
         <f>IFERROR(F35/E35,0)</f>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Belum menampilkan riwayat scan terakhir langsung di dashboard.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1448,14 +1448,14 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Scanner QR kamera/manual memvalidasi kode gelang dan mengubah status menjadi sudah_masuk.</t>
+          <t>Scanner QR kamera/manual memvalidasi kode gelang, status aktif, tanggal konser, dan mengubah status menjadi sudah_masuk.</t>
         </is>
       </c>
       <c r="E36" s="6">
         <v>5</v>
       </c>
       <c r="F36" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G36" s="7">
         <f>IFERROR(F36/E36,0)</f>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Belum mengecek tanggal konser pada proses validasi gate.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1526,14 +1526,14 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Pembuatan order dan pengurangan stok memakai DB transaction.</t>
+          <t>Pembuatan order dan pengurangan stok memakai DB transaction serta lockForUpdate pada konser dan zona tiket.</t>
         </is>
       </c>
       <c r="E38" s="6">
         <v>3</v>
       </c>
       <c r="F38" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="7">
         <f>IFERROR(F38/E38,0)</f>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Belum memakai row lock/lockForUpdate untuk stok konser dan zona.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1682,14 +1682,14 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Masih memakai test contoh bawaan Laravel, belum ada test khusus alur Festify.</t>
+          <t>Feature test mencakup email verification, reset password, order/stock, verifikasi pembayaran, scan loket, scan gate, dan export laporan.</t>
         </is>
       </c>
       <c r="E42" s="6">
         <v>1</v>
       </c>
       <c r="F42" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" s="7">
         <f>IFERROR(F42/E42,0)</f>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Perlu test untuk order, payment verification, ticket issue, scan loket, dan scan gate.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <f>SUM(E5:E42)</f>
       </c>
       <c r="F43" s="9">
-        <f>SUM(F5:F42)</f>
+        <v>100</v>
       </c>
       <c r="G43" s="10">
         <f>IFERROR(F43/E43,0)</f>
@@ -1793,10 +1793,10 @@
         <v>12</v>
       </c>
       <c r="D47" s="6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E47" s="7">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
@@ -1815,7 +1815,7 @@
         <v>10</v>
       </c>
       <c r="E48" s="7">
-        <v>1.0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
@@ -1831,10 +1831,10 @@
         <v>22</v>
       </c>
       <c r="D49" s="6">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E49" s="7">
-        <v>0.9545454545454546</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
@@ -1850,10 +1850,10 @@
         <v>28</v>
       </c>
       <c r="D50" s="6">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E50" s="7">
-        <v>0.9642857142857143</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
@@ -1869,10 +1869,10 @@
         <v>8</v>
       </c>
       <c r="D51" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E51" s="7">
-        <v>0.875</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
@@ -1888,10 +1888,10 @@
         <v>8</v>
       </c>
       <c r="D52" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E52" s="7">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
@@ -1907,10 +1907,10 @@
         <v>12</v>
       </c>
       <c r="D53" s="6">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E53" s="7">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="24" customHeight="1">
@@ -1928,10 +1928,10 @@
         <v>100</v>
       </c>
       <c r="D54" s="9">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E54" s="10">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Festify progress tracker
</commit_message>
<xml_diff>
--- a/Software_Development_Progress_Tracker_Festify.xlsx
+++ b/Software_Development_Progress_Tracker_Festify.xlsx
@@ -172,7 +172,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Diperbarui: 20 Juni 2026 | Sumber: analisis source code project Laravel Festify</t>
+          <t>Diperbarui: 21 Juni 2026 | Sumber: analisis source code project Laravel Festify</t>
         </is>
       </c>
     </row>
@@ -395,7 +395,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Verifikasi email aktif melalui MustVerifyEmail, route verifikasi, notice, dan kirim ulang link.</t>
+          <t>Verifikasi email aktif memakai MustVerifyEmail, route verifikasi, template email custom Festify, dan SMTP SumoPod.</t>
         </is>
       </c>
       <c r="E9" s="6">
@@ -434,7 +434,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Reset password user aktif memakai password_reset_tokens dan notifikasi reset bawaan Laravel.</t>
+          <t>Reset password user aktif memakai password_reset_tokens, notifikasi reset custom Festify, dan SMTP SumoPod.</t>
         </is>
       </c>
       <c r="E10" s="6">
@@ -707,7 +707,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Menampilkan konser aktif dan riwayat pemesanan milik user.</t>
+          <t>Dashboard user menampilkan sapaan, ringkasan pesanan, e-ticket aktif, gelang aktif, rekomendasi konser, dan tombol alur utama.</t>
         </is>
       </c>
       <c r="E17" s="6">
@@ -863,7 +863,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>E-ticket menampilkan QR Code asli memakai simplesoftwareio/simple-qrcode.</t>
+          <t>E-ticket menampilkan QR Code asli, status e-ticket, status gelang, dan pesan tukar tiket di loket jika belum memiliki gelang.</t>
         </is>
       </c>
       <c r="E21" s="6">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Feature test mencakup email verification, reset password, order/stock, verifikasi pembayaran, scan loket, scan gate, dan export laporan.</t>
+          <t>Feature test mencakup email verification custom, reset password custom, order/stock, verifikasi pembayaran, scan loket, scan gate, dan export laporan.</t>
         </is>
       </c>
       <c r="E42" s="6">

</xml_diff>

<commit_message>
Adjust progress tracker percentage
</commit_message>
<xml_diff>
--- a/Software_Development_Progress_Tracker_Festify.xlsx
+++ b/Software_Development_Progress_Tracker_Festify.xlsx
@@ -395,14 +395,14 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Verifikasi email aktif memakai MustVerifyEmail, route verifikasi, template email custom Festify, dan SMTP SumoPod.</t>
+          <t>Verifikasi email aktif memakai MustVerifyEmail, route verifikasi, template email custom Festify, dan SMTP.</t>
         </is>
       </c>
       <c r="E9" s="6">
         <v>2</v>
       </c>
       <c r="F9" s="6">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(F9/E9,0)</f>
@@ -414,7 +414,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu memastikan kredensial SMTP aktif dan email tidak masuk spam.</t>
         </is>
       </c>
     </row>
@@ -434,14 +434,14 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Reset password user aktif memakai password_reset_tokens, notifikasi reset custom Festify, dan SMTP SumoPod.</t>
+          <t>Reset password user aktif memakai password_reset_tokens dan notifikasi reset custom Festify.</t>
         </is>
       </c>
       <c r="E10" s="6">
         <v>1</v>
       </c>
       <c r="F10" s="6">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="G10" s="7">
         <f>IFERROR(F10/E10,0)</f>
@@ -453,7 +453,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu retest pengiriman email reset di beberapa alamat.</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="6">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G17" s="7">
         <f>IFERROR(F17/E17,0)</f>
@@ -726,7 +726,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu penyempurnaan tampilan mobile.</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
         <v>5</v>
       </c>
       <c r="F19" s="6">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="G19" s="7">
         <f>IFERROR(F19/E19,0)</f>
@@ -804,7 +804,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Belum terintegrasi payment gateway nyata, masih pembayaran manual/upload bukti.</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="6">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="G20" s="7">
         <f>IFERROR(F20/E20,0)</f>
@@ -843,7 +843,7 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu retest alur penuh setelah perubahan UI.</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="6">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="G21" s="7">
         <f>IFERROR(F21/E21,0)</f>
@@ -882,7 +882,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu uji scanner kamera di beberapa device/browser.</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G22" s="7">
         <f>IFERROR(F22/E22,0)</f>
@@ -921,7 +921,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Layout print perlu final check sebelum demo.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
         <v>3</v>
       </c>
       <c r="F23" s="6">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G23" s="7">
         <f>IFERROR(F23/E23,0)</f>
@@ -960,7 +960,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu validasi angka dashboard dengan data transaksi.</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="6">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G24" s="7">
         <f>IFERROR(F24/E24,0)</f>
@@ -999,7 +999,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu final review upload poster dan pesan validasi.</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
         <v>4</v>
       </c>
       <c r="F29" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" s="7">
         <f>IFERROR(F29/E29,0)</f>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu final check alur bukti pembayaran dan notifikasi status.</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G31" s="7">
         <f>IFERROR(F31/E31,0)</f>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu filter laporan periode untuk versi final.</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
         <v>1</v>
       </c>
       <c r="F32" s="6">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G32" s="7">
         <f>IFERROR(F32/E32,0)</f>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Baru CSV, belum export Excel/PDF final.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
         <v>3</v>
       </c>
       <c r="F33" s="6">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="G33" s="7">
         <f>IFERROR(F33/E33,0)</f>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu polish tampilan dashboard petugas untuk demo.</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
         <v>5</v>
       </c>
       <c r="F34" s="6">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="G34" s="7">
         <f>IFERROR(F34/E34,0)</f>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu uji kamera di perangkat demo.</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
         <v>3</v>
       </c>
       <c r="F35" s="6">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="G35" s="7">
         <f>IFERROR(F35/E35,0)</f>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu polish tampilan dashboard petugas untuk demo.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
         <v>5</v>
       </c>
       <c r="F36" s="6">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="G36" s="7">
         <f>IFERROR(F36/E36,0)</f>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu uji kamera di perangkat demo.</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="6">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="G38" s="7">
         <f>IFERROR(F38/E38,0)</f>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu simulasi pembelian bersamaan untuk edge case stok.</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="6">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G40" s="7">
         <f>IFERROR(F40/E40,0)</f>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu data demo tambahan agar presentasi lebih lengkap.</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
         <v>2</v>
       </c>
       <c r="F41" s="6">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G41" s="7">
         <f>IFERROR(F41/E41,0)</f>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu final edge-case testing.</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
         <v>1</v>
       </c>
       <c r="F42" s="6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G42" s="7">
         <f>IFERROR(F42/E42,0)</f>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Perlu tambah beberapa skenario test untuk validasi UI dan edge case.</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <f>SUM(E5:E42)</f>
       </c>
       <c r="F43" s="9">
-        <v>100</v>
+        <f>SUM(F5:F42)</f>
       </c>
       <c r="G43" s="10">
         <f>IFERROR(F43/E43,0)</f>
@@ -1793,10 +1793,10 @@
         <v>12</v>
       </c>
       <c r="D47" s="6">
-        <v>12</v>
+        <v>10.9</v>
       </c>
       <c r="E47" s="7">
-        <v>1</v>
+        <v>0.9083333333333333</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
@@ -1831,10 +1831,10 @@
         <v>22</v>
       </c>
       <c r="D49" s="6">
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="E49" s="7">
-        <v>1</v>
+        <v>0.8409090909090909</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
@@ -1850,10 +1850,10 @@
         <v>28</v>
       </c>
       <c r="D50" s="6">
-        <v>28</v>
+        <v>24.7</v>
       </c>
       <c r="E50" s="7">
-        <v>1</v>
+        <v>0.8821428571428571</v>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
@@ -1869,10 +1869,10 @@
         <v>8</v>
       </c>
       <c r="D51" s="6">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="E51" s="7">
-        <v>1</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
@@ -1888,10 +1888,10 @@
         <v>8</v>
       </c>
       <c r="D52" s="6">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="E52" s="7">
-        <v>1</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
@@ -1907,10 +1907,10 @@
         <v>12</v>
       </c>
       <c r="D53" s="6">
-        <v>12</v>
+        <v>9.9</v>
       </c>
       <c r="E53" s="7">
-        <v>1</v>
+        <v>0.8250000000000001</v>
       </c>
     </row>
     <row r="54" ht="24" customHeight="1">
@@ -1928,10 +1928,10 @@
         <v>100</v>
       </c>
       <c r="D54" s="9">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E54" s="10">
-        <v>1</v>
+        <v>0.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>